<commit_message>
add LOB main point
git-svn-id: http://192.168.20.11/sequoiadb/trunk@13939 6121f079-4a18-41d3-8c30-8870a322f2c2
</commit_message>
<xml_diff>
--- a/testprocess/1-process/大对象测试/【large object storage】sequoiadb-test-process.xlsx
+++ b/testprocess/1-process/大对象测试/【large object storage】sequoiadb-test-process.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="project-info" sheetId="1" r:id="rId1"/>
@@ -15,13 +15,14 @@
     <sheet name="test-report" sheetId="4" r:id="rId6"/>
     <sheet name="bug" sheetId="5" r:id="rId7"/>
     <sheet name="addendum" sheetId="7" r:id="rId8"/>
+    <sheet name="lob point" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="166">
   <si>
     <t>名称</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -624,12 +625,156 @@
     <t>测试大对象数据的性能</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>LOB关键点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1.普通表普通记录+存储大对象的文件，两者之间通过记录中的某一个字段来实现关联，从而实现一套数据库系统来实现需求，不用像MongDB使用GridFS存储大记录的方式来引入多套系统。
+2.此时对文件的管理工作，只用去对普通的记录进行管理即可，如冗余，分区以及备份。
+3.大对象表必须依附于普通表存在，一个表中的大对象不能被另外一个表访问。
+4.当用户上传一个大对象时，首先生成一个全局唯一的描述符，同时我们将其按照256KB(默认)大小切片。最后按照描述符+切片id进行hash，用于决定存在哪个数据组中。
+5.大对象表所在的数据组的范围与对应的普通表的范围相同。比如有foo.bar在数据组1,2,3上，这时大对象表同样在这三个数据组上按照描述符+切片id进行hash分区。注意此时普通表的分区键并不作用于大对象表。
+6.当用户读取大对象时，我们按照其元数据+offset+len进行计算在哪个切片上，最后将数据节点返回的数据按顺序排列返回客户端。【切片存储，是为了更快的存储】【直接在数据库上对mp3等数据进行操作】
+7.由于我们是将文件切片存储，一个文件可能有非常多个分片，所以在访问的时候coord需要提供请求合并的机制，防止访问一个对象时coord需要向data发送成千上万此请求。
+8.LOB必须依赖于普通的collection。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">typedef INT32 (*)( void *, UINT32 bufLen, CHAR *buf, UINT32 &amp;len ) sdbLobWrite;
+INT32 sdbPutLobFromFunc(sdbCollectionHandle, sdbLobWrite , sdbLobHandle *);
+INT32 sdbPutLobFromFile(sdbCollectionHandle , const CHAR *fullPath , sdbLobHandle *) ;
+INT32 sdbGenLobKey( oid &amp; ) ;
+INT32 sdbOpenLob(sdbCollectionHandle , const oid *, INT32 mode, sdbLobHandle* );
+INT32 sdbReadLob(sdbLobHandle, const CHAR **out, UINT32 *len) ;
+INT32 sdbWriteLob(sdbLobHandle, const CHAR *buf, UINT32 len);
+INT32 sdbSeekLob(sdbLobHandle, UINT64 offset, LOB_SEEK whence ) ;
+INT32 sdbRemoveLob( const oid *);
+INT32 sdbCloseLob (sdbLobHandle);
+INT32 sdbLob2Bson(sdbLobHandle, bson *);
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>var fileid = db.foo.bar.putLob('/opt/xxx.avi');
+db.foo.bar.insert({filename:'xxx.avi',
+               link:'www.sequoiadb.com/a/b/c/d',
+               file:fildid.toObj ()});
+var c = db.foo.bar.getLob(fileid, "/opt/xxx.avi 2");
+db.foo.bar.dropLob(fileid);
+db.foo.bar.remove({file:fileid.toObj()})</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sdb shell示例</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C驱动接口</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LOB 测试要点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>遗留的问题</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>删除记录时自动删除关联</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>lob</t>
+    </r>
+  </si>
+  <si>
+    <t>上传未完成时意外中断自动回滚数据</t>
+  </si>
+  <si>
+    <r>
+      <t>有没有必要以树的方式处理</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>hash</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>冲突</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>dps</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>结构和同步流程</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>split</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>流程</t>
+    </r>
+  </si>
+  <si>
+    <t>备份流程</t>
+  </si>
+  <si>
+    <t>数据文件重组</t>
+  </si>
+  <si>
+    <t>全量恢复</t>
+  </si>
+  <si>
+    <t>数据回滚</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -698,8 +843,47 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="黑体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="楷体_GB2312"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFFFF00"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -778,8 +962,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="41">
+  <borders count="53">
     <border>
       <left/>
       <right/>
@@ -1297,11 +1487,145 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1498,6 +1822,66 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1549,69 +1933,9 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1620,6 +1944,78 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2133,240 +2529,240 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:20" ht="22.5" customHeight="1">
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="78" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
     </row>
     <row r="3" spans="2:20" ht="14.25" thickBot="1">
-      <c r="B3" s="102" t="s">
+      <c r="B3" s="79" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
-      <c r="Q3" s="102"/>
-      <c r="R3" s="102"/>
+      <c r="C3" s="79"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="79"/>
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+      <c r="J3" s="79"/>
+      <c r="K3" s="79"/>
+      <c r="L3" s="79"/>
+      <c r="M3" s="79"/>
+      <c r="N3" s="79"/>
+      <c r="O3" s="79"/>
+      <c r="P3" s="79"/>
+      <c r="Q3" s="79"/>
+      <c r="R3" s="79"/>
     </row>
     <row r="4" spans="2:20" ht="13.5" customHeight="1">
-      <c r="B4" s="96" t="s">
+      <c r="B4" s="89" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="106" t="s">
+      <c r="C4" s="82" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="103" t="s">
+      <c r="D4" s="80" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="103"/>
-      <c r="F4" s="103"/>
-      <c r="G4" s="99" t="s">
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="72" t="s">
         <v>147</v>
       </c>
-      <c r="H4" s="99"/>
-      <c r="I4" s="99"/>
-      <c r="J4" s="99"/>
-      <c r="K4" s="99"/>
-      <c r="L4" s="99"/>
-      <c r="M4" s="99"/>
-      <c r="N4" s="99"/>
-      <c r="O4" s="99"/>
-      <c r="P4" s="99"/>
-      <c r="Q4" s="99"/>
-      <c r="R4" s="103" t="s">
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
+      <c r="L4" s="72"/>
+      <c r="M4" s="72"/>
+      <c r="N4" s="72"/>
+      <c r="O4" s="72"/>
+      <c r="P4" s="72"/>
+      <c r="Q4" s="72"/>
+      <c r="R4" s="80" t="s">
         <v>40</v>
       </c>
-      <c r="S4" s="103"/>
-      <c r="T4" s="104"/>
+      <c r="S4" s="80"/>
+      <c r="T4" s="81"/>
     </row>
     <row r="5" spans="2:20">
-      <c r="B5" s="97"/>
-      <c r="C5" s="107"/>
-      <c r="D5" s="99"/>
-      <c r="E5" s="99"/>
-      <c r="F5" s="99"/>
-      <c r="G5" s="99"/>
-      <c r="H5" s="99"/>
-      <c r="I5" s="99"/>
-      <c r="J5" s="99"/>
-      <c r="K5" s="99"/>
-      <c r="L5" s="99"/>
-      <c r="M5" s="99"/>
-      <c r="N5" s="99"/>
-      <c r="O5" s="99"/>
-      <c r="P5" s="99"/>
-      <c r="Q5" s="99"/>
-      <c r="R5" s="99"/>
-      <c r="S5" s="99"/>
-      <c r="T5" s="105"/>
+      <c r="B5" s="90"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="72"/>
+      <c r="H5" s="72"/>
+      <c r="I5" s="72"/>
+      <c r="J5" s="72"/>
+      <c r="K5" s="72"/>
+      <c r="L5" s="72"/>
+      <c r="M5" s="72"/>
+      <c r="N5" s="72"/>
+      <c r="O5" s="72"/>
+      <c r="P5" s="72"/>
+      <c r="Q5" s="72"/>
+      <c r="R5" s="72"/>
+      <c r="S5" s="72"/>
+      <c r="T5" s="73"/>
     </row>
     <row r="6" spans="2:20">
-      <c r="B6" s="97"/>
-      <c r="C6" s="107" t="s">
+      <c r="B6" s="90"/>
+      <c r="C6" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="D6" s="99" t="s">
+      <c r="D6" s="72" t="s">
         <v>139</v>
       </c>
-      <c r="E6" s="99"/>
-      <c r="F6" s="99"/>
-      <c r="G6" s="99"/>
-      <c r="H6" s="99"/>
-      <c r="I6" s="99"/>
-      <c r="J6" s="99"/>
-      <c r="K6" s="99"/>
-      <c r="L6" s="99"/>
-      <c r="M6" s="99"/>
-      <c r="N6" s="99"/>
-      <c r="O6" s="99"/>
-      <c r="P6" s="99"/>
-      <c r="Q6" s="99"/>
-      <c r="R6" s="99" t="s">
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="72"/>
+      <c r="J6" s="72"/>
+      <c r="K6" s="72"/>
+      <c r="L6" s="72"/>
+      <c r="M6" s="72"/>
+      <c r="N6" s="72"/>
+      <c r="O6" s="72"/>
+      <c r="P6" s="72"/>
+      <c r="Q6" s="72"/>
+      <c r="R6" s="72" t="s">
         <v>36</v>
       </c>
-      <c r="S6" s="99"/>
-      <c r="T6" s="105"/>
+      <c r="S6" s="72"/>
+      <c r="T6" s="73"/>
     </row>
     <row r="7" spans="2:20">
-      <c r="B7" s="97"/>
-      <c r="C7" s="107"/>
-      <c r="D7" s="99"/>
-      <c r="E7" s="99"/>
-      <c r="F7" s="99"/>
-      <c r="G7" s="99"/>
-      <c r="H7" s="99"/>
-      <c r="I7" s="99"/>
-      <c r="J7" s="99"/>
-      <c r="K7" s="99"/>
-      <c r="L7" s="99"/>
-      <c r="M7" s="99"/>
-      <c r="N7" s="99"/>
-      <c r="O7" s="99"/>
-      <c r="P7" s="99"/>
-      <c r="Q7" s="99"/>
-      <c r="R7" s="99"/>
-      <c r="S7" s="99"/>
-      <c r="T7" s="105"/>
+      <c r="B7" s="90"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="72"/>
+      <c r="E7" s="72"/>
+      <c r="F7" s="72"/>
+      <c r="G7" s="72"/>
+      <c r="H7" s="72"/>
+      <c r="I7" s="72"/>
+      <c r="J7" s="72"/>
+      <c r="K7" s="72"/>
+      <c r="L7" s="72"/>
+      <c r="M7" s="72"/>
+      <c r="N7" s="72"/>
+      <c r="O7" s="72"/>
+      <c r="P7" s="72"/>
+      <c r="Q7" s="72"/>
+      <c r="R7" s="72"/>
+      <c r="S7" s="72"/>
+      <c r="T7" s="73"/>
     </row>
     <row r="8" spans="2:20" ht="13.5" customHeight="1">
-      <c r="B8" s="97"/>
-      <c r="C8" s="107" t="s">
+      <c r="B8" s="90"/>
+      <c r="C8" s="76" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="99" t="s">
+      <c r="D8" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="E8" s="99"/>
-      <c r="F8" s="99"/>
-      <c r="G8" s="76"/>
-      <c r="H8" s="77"/>
-      <c r="I8" s="77"/>
-      <c r="J8" s="77"/>
-      <c r="K8" s="77"/>
-      <c r="L8" s="77"/>
-      <c r="M8" s="77"/>
-      <c r="N8" s="77"/>
-      <c r="O8" s="77"/>
-      <c r="P8" s="77"/>
-      <c r="Q8" s="78"/>
-      <c r="R8" s="99"/>
-      <c r="S8" s="99"/>
-      <c r="T8" s="105"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="96"/>
+      <c r="H8" s="97"/>
+      <c r="I8" s="97"/>
+      <c r="J8" s="97"/>
+      <c r="K8" s="97"/>
+      <c r="L8" s="97"/>
+      <c r="M8" s="97"/>
+      <c r="N8" s="97"/>
+      <c r="O8" s="97"/>
+      <c r="P8" s="97"/>
+      <c r="Q8" s="98"/>
+      <c r="R8" s="72"/>
+      <c r="S8" s="72"/>
+      <c r="T8" s="73"/>
     </row>
     <row r="9" spans="2:20">
-      <c r="B9" s="97"/>
-      <c r="C9" s="107"/>
-      <c r="D9" s="99"/>
-      <c r="E9" s="99"/>
-      <c r="F9" s="99"/>
-      <c r="G9" s="79"/>
-      <c r="H9" s="80"/>
-      <c r="I9" s="80"/>
-      <c r="J9" s="80"/>
-      <c r="K9" s="80"/>
-      <c r="L9" s="80"/>
-      <c r="M9" s="80"/>
-      <c r="N9" s="80"/>
-      <c r="O9" s="80"/>
-      <c r="P9" s="80"/>
-      <c r="Q9" s="81"/>
-      <c r="R9" s="99"/>
-      <c r="S9" s="99"/>
-      <c r="T9" s="105"/>
+      <c r="B9" s="90"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="72"/>
+      <c r="F9" s="72"/>
+      <c r="G9" s="99"/>
+      <c r="H9" s="100"/>
+      <c r="I9" s="100"/>
+      <c r="J9" s="100"/>
+      <c r="K9" s="100"/>
+      <c r="L9" s="100"/>
+      <c r="M9" s="100"/>
+      <c r="N9" s="100"/>
+      <c r="O9" s="100"/>
+      <c r="P9" s="100"/>
+      <c r="Q9" s="101"/>
+      <c r="R9" s="72"/>
+      <c r="S9" s="72"/>
+      <c r="T9" s="73"/>
     </row>
     <row r="10" spans="2:20">
-      <c r="B10" s="97"/>
-      <c r="C10" s="107" t="s">
+      <c r="B10" s="90"/>
+      <c r="C10" s="76" t="s">
         <v>106</v>
       </c>
-      <c r="D10" s="99" t="s">
+      <c r="D10" s="72" t="s">
         <v>148</v>
       </c>
-      <c r="E10" s="99"/>
-      <c r="F10" s="99"/>
-      <c r="G10" s="82"/>
-      <c r="H10" s="83"/>
-      <c r="I10" s="83"/>
-      <c r="J10" s="83"/>
-      <c r="K10" s="83"/>
-      <c r="L10" s="83"/>
-      <c r="M10" s="83"/>
-      <c r="N10" s="83"/>
-      <c r="O10" s="83"/>
-      <c r="P10" s="83"/>
-      <c r="Q10" s="84"/>
-      <c r="R10" s="99"/>
-      <c r="S10" s="99"/>
-      <c r="T10" s="105"/>
+      <c r="E10" s="72"/>
+      <c r="F10" s="72"/>
+      <c r="G10" s="102"/>
+      <c r="H10" s="103"/>
+      <c r="I10" s="103"/>
+      <c r="J10" s="103"/>
+      <c r="K10" s="103"/>
+      <c r="L10" s="103"/>
+      <c r="M10" s="103"/>
+      <c r="N10" s="103"/>
+      <c r="O10" s="103"/>
+      <c r="P10" s="103"/>
+      <c r="Q10" s="104"/>
+      <c r="R10" s="72"/>
+      <c r="S10" s="72"/>
+      <c r="T10" s="73"/>
     </row>
     <row r="11" spans="2:20" ht="14.25" thickBot="1">
-      <c r="B11" s="98"/>
-      <c r="C11" s="109"/>
-      <c r="D11" s="100"/>
-      <c r="E11" s="100"/>
-      <c r="F11" s="100"/>
-      <c r="G11" s="85"/>
-      <c r="H11" s="86"/>
-      <c r="I11" s="86"/>
-      <c r="J11" s="86"/>
-      <c r="K11" s="86"/>
-      <c r="L11" s="86"/>
-      <c r="M11" s="86"/>
-      <c r="N11" s="86"/>
-      <c r="O11" s="86"/>
-      <c r="P11" s="86"/>
-      <c r="Q11" s="87"/>
-      <c r="R11" s="100"/>
-      <c r="S11" s="100"/>
-      <c r="T11" s="108"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="105"/>
+      <c r="H11" s="106"/>
+      <c r="I11" s="106"/>
+      <c r="J11" s="106"/>
+      <c r="K11" s="106"/>
+      <c r="L11" s="106"/>
+      <c r="M11" s="106"/>
+      <c r="N11" s="106"/>
+      <c r="O11" s="106"/>
+      <c r="P11" s="106"/>
+      <c r="Q11" s="107"/>
+      <c r="R11" s="74"/>
+      <c r="S11" s="74"/>
+      <c r="T11" s="75"/>
     </row>
     <row r="15" spans="2:20" ht="14.25" thickBot="1"/>
     <row r="16" spans="2:20" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B16" s="91" t="s">
+      <c r="B16" s="83" t="s">
         <v>47</v>
       </c>
       <c r="C16" s="51"/>
@@ -2393,7 +2789,7 @@
       </c>
     </row>
     <row r="17" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B17" s="92"/>
+      <c r="B17" s="84"/>
       <c r="C17" s="51" t="s">
         <v>112</v>
       </c>
@@ -2420,7 +2816,7 @@
       </c>
     </row>
     <row r="18" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B18" s="92"/>
+      <c r="B18" s="84"/>
       <c r="C18" s="51" t="s">
         <v>113</v>
       </c>
@@ -2447,7 +2843,7 @@
       </c>
     </row>
     <row r="19" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B19" s="92"/>
+      <c r="B19" s="84"/>
       <c r="C19" s="51" t="s">
         <v>114</v>
       </c>
@@ -2474,7 +2870,7 @@
       </c>
     </row>
     <row r="20" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B20" s="92"/>
+      <c r="B20" s="84"/>
       <c r="C20" s="51" t="s">
         <v>141</v>
       </c>
@@ -2501,7 +2897,7 @@
       </c>
     </row>
     <row r="21" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B21" s="92"/>
+      <c r="B21" s="84"/>
       <c r="C21" s="51" t="s">
         <v>115</v>
       </c>
@@ -2528,7 +2924,7 @@
       </c>
     </row>
     <row r="22" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B22" s="92"/>
+      <c r="B22" s="84"/>
       <c r="C22" s="51" t="s">
         <v>116</v>
       </c>
@@ -2555,7 +2951,7 @@
       </c>
     </row>
     <row r="23" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B23" s="92"/>
+      <c r="B23" s="84"/>
       <c r="C23" s="51" t="s">
         <v>117</v>
       </c>
@@ -2582,7 +2978,7 @@
       </c>
     </row>
     <row r="24" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B24" s="92"/>
+      <c r="B24" s="84"/>
       <c r="C24" s="51" t="s">
         <v>118</v>
       </c>
@@ -2609,7 +3005,7 @@
       </c>
     </row>
     <row r="25" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B25" s="92"/>
+      <c r="B25" s="84"/>
       <c r="C25" s="51"/>
       <c r="D25" s="48"/>
       <c r="E25" s="33"/>
@@ -2622,24 +3018,24 @@
       <c r="L25" s="41"/>
     </row>
     <row r="26" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B26" s="92"/>
+      <c r="B26" s="84"/>
       <c r="C26" s="51" t="s">
         <v>145</v>
       </c>
-      <c r="D26" s="88" t="s">
+      <c r="D26" s="108" t="s">
         <v>146</v>
       </c>
-      <c r="E26" s="89"/>
-      <c r="F26" s="89"/>
-      <c r="G26" s="89"/>
-      <c r="H26" s="89"/>
-      <c r="I26" s="89"/>
-      <c r="J26" s="89"/>
-      <c r="K26" s="90"/>
+      <c r="E26" s="87"/>
+      <c r="F26" s="87"/>
+      <c r="G26" s="87"/>
+      <c r="H26" s="87"/>
+      <c r="I26" s="87"/>
+      <c r="J26" s="87"/>
+      <c r="K26" s="109"/>
       <c r="L26" s="41"/>
     </row>
     <row r="27" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B27" s="93"/>
+      <c r="B27" s="85"/>
       <c r="C27" s="52"/>
       <c r="D27" s="50"/>
       <c r="E27" s="34"/>
@@ -2653,7 +3049,7 @@
     </row>
     <row r="31" spans="2:12" ht="14.25" thickBot="1"/>
     <row r="32" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B32" s="91" t="s">
+      <c r="B32" s="83" t="s">
         <v>49</v>
       </c>
       <c r="C32" s="51"/>
@@ -2686,7 +3082,7 @@
       </c>
     </row>
     <row r="33" spans="2:13" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B33" s="92"/>
+      <c r="B33" s="84"/>
       <c r="C33" s="56" t="s">
         <v>50</v>
       </c>
@@ -2717,12 +3113,12 @@
       <c r="L33" s="41" t="s">
         <v>121</v>
       </c>
-      <c r="M33" s="72" t="s">
+      <c r="M33" s="92" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="34" spans="2:13" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B34" s="92"/>
+      <c r="B34" s="84"/>
       <c r="C34" s="56" t="s">
         <v>95</v>
       </c>
@@ -2753,10 +3149,10 @@
       <c r="L34" s="41" t="s">
         <v>122</v>
       </c>
-      <c r="M34" s="72"/>
+      <c r="M34" s="92"/>
     </row>
     <row r="35" spans="2:13" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B35" s="92"/>
+      <c r="B35" s="84"/>
       <c r="C35" s="56" t="s">
         <v>96</v>
       </c>
@@ -2787,10 +3183,10 @@
       <c r="L35" s="41" t="s">
         <v>123</v>
       </c>
-      <c r="M35" s="72"/>
+      <c r="M35" s="92"/>
     </row>
     <row r="36" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B36" s="92"/>
+      <c r="B36" s="84"/>
       <c r="C36" s="57" t="s">
         <v>51</v>
       </c>
@@ -2819,12 +3215,12 @@
       <c r="L36" s="41" t="s">
         <v>124</v>
       </c>
-      <c r="M36" s="73" t="s">
+      <c r="M36" s="93" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="37" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B37" s="92"/>
+      <c r="B37" s="84"/>
       <c r="C37" s="57" t="s">
         <v>97</v>
       </c>
@@ -2853,10 +3249,10 @@
       <c r="L37" s="41" t="s">
         <v>122</v>
       </c>
-      <c r="M37" s="73"/>
+      <c r="M37" s="93"/>
     </row>
     <row r="38" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B38" s="92"/>
+      <c r="B38" s="84"/>
       <c r="C38" s="57" t="s">
         <v>98</v>
       </c>
@@ -2885,10 +3281,10 @@
       <c r="L38" s="41" t="s">
         <v>125</v>
       </c>
-      <c r="M38" s="73"/>
+      <c r="M38" s="93"/>
     </row>
     <row r="39" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B39" s="92"/>
+      <c r="B39" s="84"/>
       <c r="C39" s="55" t="s">
         <v>55</v>
       </c>
@@ -2917,12 +3313,12 @@
       <c r="L39" s="41" t="s">
         <v>126</v>
       </c>
-      <c r="M39" s="74" t="s">
+      <c r="M39" s="94" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="40" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B40" s="92"/>
+      <c r="B40" s="84"/>
       <c r="C40" s="55" t="s">
         <v>90</v>
       </c>
@@ -2951,10 +3347,10 @@
       <c r="L40" s="41" t="s">
         <v>127</v>
       </c>
-      <c r="M40" s="74"/>
+      <c r="M40" s="94"/>
     </row>
     <row r="41" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B41" s="92"/>
+      <c r="B41" s="84"/>
       <c r="C41" s="55" t="s">
         <v>91</v>
       </c>
@@ -2983,10 +3379,10 @@
       <c r="L41" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="M41" s="74"/>
+      <c r="M41" s="94"/>
     </row>
     <row r="42" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B42" s="92"/>
+      <c r="B42" s="84"/>
       <c r="C42" s="58" t="s">
         <v>56</v>
       </c>
@@ -3015,12 +3411,12 @@
       <c r="L42" s="41" t="s">
         <v>129</v>
       </c>
-      <c r="M42" s="75" t="s">
+      <c r="M42" s="95" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="43" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B43" s="92"/>
+      <c r="B43" s="84"/>
       <c r="C43" s="58" t="s">
         <v>102</v>
       </c>
@@ -3049,10 +3445,10 @@
       <c r="L43" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="M43" s="75"/>
+      <c r="M43" s="95"/>
     </row>
     <row r="44" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B44" s="92"/>
+      <c r="B44" s="84"/>
       <c r="C44" s="58" t="s">
         <v>57</v>
       </c>
@@ -3081,10 +3477,10 @@
       <c r="L44" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="M44" s="75"/>
+      <c r="M44" s="95"/>
     </row>
     <row r="45" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B45" s="92"/>
+      <c r="B45" s="84"/>
       <c r="C45" s="59" t="s">
         <v>92</v>
       </c>
@@ -3115,7 +3511,7 @@
       </c>
     </row>
     <row r="46" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B46" s="92"/>
+      <c r="B46" s="84"/>
       <c r="C46" s="59" t="s">
         <v>132</v>
       </c>
@@ -3146,7 +3542,7 @@
       </c>
     </row>
     <row r="47" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B47" s="92"/>
+      <c r="B47" s="84"/>
       <c r="C47" s="59" t="s">
         <v>93</v>
       </c>
@@ -3177,7 +3573,7 @@
       </c>
     </row>
     <row r="48" spans="2:13" ht="14.25" thickBot="1">
-      <c r="B48" s="92"/>
+      <c r="B48" s="84"/>
       <c r="C48" s="60" t="s">
         <v>100</v>
       </c>
@@ -3208,7 +3604,7 @@
       </c>
     </row>
     <row r="49" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B49" s="92"/>
+      <c r="B49" s="84"/>
       <c r="C49" s="60" t="s">
         <v>101</v>
       </c>
@@ -3239,7 +3635,7 @@
       </c>
     </row>
     <row r="50" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B50" s="92"/>
+      <c r="B50" s="84"/>
       <c r="C50" s="62" t="s">
         <v>142</v>
       </c>
@@ -3268,7 +3664,7 @@
       <c r="L50" s="41"/>
     </row>
     <row r="51" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B51" s="92"/>
+      <c r="B51" s="84"/>
       <c r="C51" s="63" t="s">
         <v>143</v>
       </c>
@@ -3297,7 +3693,7 @@
       <c r="L51" s="46"/>
     </row>
     <row r="52" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B52" s="92"/>
+      <c r="B52" s="84"/>
       <c r="C52" s="63" t="s">
         <v>144</v>
       </c>
@@ -3326,7 +3722,7 @@
       <c r="L52" s="46"/>
     </row>
     <row r="53" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B53" s="93"/>
+      <c r="B53" s="85"/>
       <c r="C53" s="52"/>
       <c r="D53" s="50"/>
       <c r="E53" s="34"/>
@@ -3340,7 +3736,7 @@
     </row>
     <row r="57" spans="2:12" ht="14.25" thickBot="1"/>
     <row r="58" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B58" s="91" t="s">
+      <c r="B58" s="83" t="s">
         <v>58</v>
       </c>
       <c r="C58" s="51"/>
@@ -3371,7 +3767,7 @@
       </c>
     </row>
     <row r="59" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B59" s="92"/>
+      <c r="B59" s="84"/>
       <c r="C59" s="51" t="s">
         <v>64</v>
       </c>
@@ -3402,7 +3798,7 @@
       </c>
     </row>
     <row r="60" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B60" s="92"/>
+      <c r="B60" s="84"/>
       <c r="C60" s="51" t="s">
         <v>65</v>
       </c>
@@ -3433,7 +3829,7 @@
       </c>
     </row>
     <row r="61" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B61" s="92"/>
+      <c r="B61" s="84"/>
       <c r="C61" s="51" t="s">
         <v>67</v>
       </c>
@@ -3464,7 +3860,7 @@
       </c>
     </row>
     <row r="62" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B62" s="92"/>
+      <c r="B62" s="84"/>
       <c r="C62" s="51" t="s">
         <v>69</v>
       </c>
@@ -3495,7 +3891,7 @@
       </c>
     </row>
     <row r="63" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B63" s="92"/>
+      <c r="B63" s="84"/>
       <c r="C63" s="51" t="s">
         <v>71</v>
       </c>
@@ -3526,7 +3922,7 @@
       </c>
     </row>
     <row r="64" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B64" s="92"/>
+      <c r="B64" s="84"/>
       <c r="C64" s="51" t="s">
         <v>72</v>
       </c>
@@ -3557,7 +3953,7 @@
       </c>
     </row>
     <row r="65" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B65" s="92"/>
+      <c r="B65" s="84"/>
       <c r="C65" s="51" t="s">
         <v>73</v>
       </c>
@@ -3588,7 +3984,7 @@
       </c>
     </row>
     <row r="66" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B66" s="92"/>
+      <c r="B66" s="84"/>
       <c r="C66" s="51" t="s">
         <v>74</v>
       </c>
@@ -3619,7 +4015,7 @@
       </c>
     </row>
     <row r="67" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B67" s="92"/>
+      <c r="B67" s="84"/>
       <c r="C67" s="51"/>
       <c r="D67" s="48"/>
       <c r="E67" s="33"/>
@@ -3632,7 +4028,7 @@
       <c r="L67" s="41"/>
     </row>
     <row r="68" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B68" s="92"/>
+      <c r="B68" s="84"/>
       <c r="C68" s="51"/>
       <c r="D68" s="48"/>
       <c r="E68" s="33"/>
@@ -3645,7 +4041,7 @@
       <c r="L68" s="41"/>
     </row>
     <row r="69" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B69" s="93"/>
+      <c r="B69" s="85"/>
       <c r="C69" s="52"/>
       <c r="D69" s="50"/>
       <c r="E69" s="34"/>
@@ -3659,7 +4055,7 @@
     </row>
     <row r="73" spans="2:12" ht="14.25" thickBot="1"/>
     <row r="74" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B74" s="91" t="s">
+      <c r="B74" s="83" t="s">
         <v>80</v>
       </c>
       <c r="C74" s="51"/>
@@ -3690,7 +4086,7 @@
       </c>
     </row>
     <row r="75" spans="2:12" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B75" s="92"/>
+      <c r="B75" s="84"/>
       <c r="C75" s="51" t="s">
         <v>81</v>
       </c>
@@ -3717,7 +4113,7 @@
       </c>
     </row>
     <row r="76" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B76" s="92"/>
+      <c r="B76" s="84"/>
       <c r="C76" s="51" t="s">
         <v>82</v>
       </c>
@@ -3744,7 +4140,7 @@
       </c>
     </row>
     <row r="77" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B77" s="92"/>
+      <c r="B77" s="84"/>
       <c r="C77" s="51" t="s">
         <v>83</v>
       </c>
@@ -3771,7 +4167,7 @@
       </c>
     </row>
     <row r="78" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B78" s="92"/>
+      <c r="B78" s="84"/>
       <c r="C78" s="51" t="s">
         <v>84</v>
       </c>
@@ -3798,7 +4194,7 @@
       </c>
     </row>
     <row r="79" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B79" s="92"/>
+      <c r="B79" s="84"/>
       <c r="C79" s="51" t="s">
         <v>81</v>
       </c>
@@ -3825,7 +4221,7 @@
       </c>
     </row>
     <row r="80" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B80" s="92"/>
+      <c r="B80" s="84"/>
       <c r="C80" s="51" t="s">
         <v>82</v>
       </c>
@@ -3852,7 +4248,7 @@
       </c>
     </row>
     <row r="81" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B81" s="92"/>
+      <c r="B81" s="84"/>
       <c r="C81" s="51" t="s">
         <v>83</v>
       </c>
@@ -3879,7 +4275,7 @@
       </c>
     </row>
     <row r="82" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B82" s="92"/>
+      <c r="B82" s="84"/>
       <c r="C82" s="51" t="s">
         <v>84</v>
       </c>
@@ -3906,7 +4302,7 @@
       </c>
     </row>
     <row r="83" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B83" s="92"/>
+      <c r="B83" s="84"/>
       <c r="C83" s="51"/>
       <c r="D83" s="48"/>
       <c r="E83" s="33"/>
@@ -3919,22 +4315,22 @@
       <c r="L83" s="46"/>
     </row>
     <row r="84" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B84" s="92"/>
+      <c r="B84" s="84"/>
       <c r="C84" s="53"/>
       <c r="D84" s="49"/>
       <c r="E84" s="38"/>
       <c r="F84" s="38"/>
-      <c r="G84" s="94" t="s">
+      <c r="G84" s="86" t="s">
         <v>137</v>
       </c>
-      <c r="H84" s="89"/>
-      <c r="I84" s="95"/>
+      <c r="H84" s="87"/>
+      <c r="I84" s="88"/>
       <c r="J84" s="61"/>
       <c r="K84" s="44"/>
       <c r="L84" s="46"/>
     </row>
     <row r="85" spans="2:12" ht="14.25" thickBot="1">
-      <c r="B85" s="93"/>
+      <c r="B85" s="85"/>
       <c r="C85" s="52"/>
       <c r="D85" s="50"/>
       <c r="E85" s="34"/>
@@ -3948,12 +4344,21 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="R8:T9"/>
-    <mergeCell ref="R10:T11"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="G4:Q5"/>
-    <mergeCell ref="G6:Q7"/>
+    <mergeCell ref="M33:M35"/>
+    <mergeCell ref="M36:M38"/>
+    <mergeCell ref="M39:M41"/>
+    <mergeCell ref="M42:M44"/>
+    <mergeCell ref="G8:Q9"/>
+    <mergeCell ref="G10:Q11"/>
+    <mergeCell ref="D26:K26"/>
+    <mergeCell ref="B32:B53"/>
+    <mergeCell ref="B58:B69"/>
+    <mergeCell ref="B74:B85"/>
+    <mergeCell ref="G84:I84"/>
+    <mergeCell ref="B4:B11"/>
+    <mergeCell ref="B16:B27"/>
+    <mergeCell ref="D8:F9"/>
+    <mergeCell ref="D10:F11"/>
     <mergeCell ref="B1:P1"/>
     <mergeCell ref="B3:R3"/>
     <mergeCell ref="D4:F5"/>
@@ -3962,21 +4367,12 @@
     <mergeCell ref="R6:T7"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="C6:C7"/>
-    <mergeCell ref="B32:B53"/>
-    <mergeCell ref="B58:B69"/>
-    <mergeCell ref="B74:B85"/>
-    <mergeCell ref="G84:I84"/>
-    <mergeCell ref="B4:B11"/>
-    <mergeCell ref="B16:B27"/>
-    <mergeCell ref="D8:F9"/>
-    <mergeCell ref="D10:F11"/>
-    <mergeCell ref="M33:M35"/>
-    <mergeCell ref="M36:M38"/>
-    <mergeCell ref="M39:M41"/>
-    <mergeCell ref="M42:M44"/>
-    <mergeCell ref="G8:Q9"/>
-    <mergeCell ref="G10:Q11"/>
-    <mergeCell ref="D26:K26"/>
+    <mergeCell ref="R8:T9"/>
+    <mergeCell ref="R10:T11"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="G4:Q5"/>
+    <mergeCell ref="G6:Q7"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4029,18 +4425,18 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
-      <c r="F4" s="101" t="s">
+      <c r="F4" s="78" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="101"/>
+      <c r="G4" s="78"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="F5" s="101"/>
-      <c r="G5" s="101"/>
+      <c r="F5" s="78"/>
+      <c r="G5" s="78"/>
     </row>
     <row r="6" spans="1:7">
-      <c r="F6" s="101"/>
-      <c r="G6" s="101"/>
+      <c r="F6" s="78"/>
+      <c r="G6" s="78"/>
     </row>
     <row r="7" spans="1:7">
       <c r="B7"/>
@@ -4825,9 +5221,825 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="B2:B12"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="42.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2" ht="14.25" thickBot="1"/>
+    <row r="3" spans="2:2" ht="23.25" thickBot="1">
+      <c r="B3" s="132" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" ht="20.25" thickBot="1">
+      <c r="B4" s="133" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" ht="24" customHeight="1" thickBot="1">
+      <c r="B5" s="134" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" ht="21" customHeight="1" thickBot="1">
+      <c r="B6" s="134" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" ht="20.25" thickBot="1">
+      <c r="B7" s="135" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" ht="20.25" thickBot="1">
+      <c r="B8" s="135" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" ht="19.5" thickBot="1">
+      <c r="B9" s="134" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" ht="19.5" thickBot="1">
+      <c r="B10" s="134" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" ht="19.5" thickBot="1">
+      <c r="B11" s="134" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" ht="19.5" thickBot="1">
+      <c r="B12" s="136" t="s">
+        <v>165</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="B2:V34"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
+  <cols>
+    <col min="1" max="1" width="3.125" customWidth="1"/>
+    <col min="2" max="2" width="9.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:22" ht="25.5">
+      <c r="H2" s="131" t="s">
+        <v>155</v>
+      </c>
+      <c r="I2" s="131"/>
+      <c r="J2" s="131"/>
+      <c r="K2" s="131"/>
+      <c r="L2" s="131"/>
+      <c r="M2" s="131"/>
+      <c r="N2" s="131"/>
+    </row>
+    <row r="3" spans="2:22" ht="14.25" thickBot="1"/>
+    <row r="4" spans="2:22">
+      <c r="B4" s="113" t="s">
+        <v>149</v>
+      </c>
+      <c r="C4" s="116" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" s="117"/>
+      <c r="E4" s="117"/>
+      <c r="F4" s="117"/>
+      <c r="G4" s="117"/>
+      <c r="H4" s="117"/>
+      <c r="I4" s="117"/>
+      <c r="J4" s="117"/>
+      <c r="K4" s="117"/>
+      <c r="L4" s="117"/>
+      <c r="M4" s="117"/>
+      <c r="N4" s="117"/>
+      <c r="O4" s="117"/>
+      <c r="P4" s="117"/>
+      <c r="Q4" s="117"/>
+      <c r="R4" s="117"/>
+      <c r="S4" s="117"/>
+      <c r="T4" s="117"/>
+      <c r="U4" s="117"/>
+      <c r="V4" s="118"/>
+    </row>
+    <row r="5" spans="2:22">
+      <c r="B5" s="114"/>
+      <c r="C5" s="119"/>
+      <c r="D5" s="120"/>
+      <c r="E5" s="120"/>
+      <c r="F5" s="120"/>
+      <c r="G5" s="120"/>
+      <c r="H5" s="120"/>
+      <c r="I5" s="120"/>
+      <c r="J5" s="120"/>
+      <c r="K5" s="120"/>
+      <c r="L5" s="120"/>
+      <c r="M5" s="120"/>
+      <c r="N5" s="120"/>
+      <c r="O5" s="120"/>
+      <c r="P5" s="120"/>
+      <c r="Q5" s="120"/>
+      <c r="R5" s="120"/>
+      <c r="S5" s="120"/>
+      <c r="T5" s="120"/>
+      <c r="U5" s="120"/>
+      <c r="V5" s="121"/>
+    </row>
+    <row r="6" spans="2:22">
+      <c r="B6" s="114"/>
+      <c r="C6" s="119"/>
+      <c r="D6" s="120"/>
+      <c r="E6" s="120"/>
+      <c r="F6" s="120"/>
+      <c r="G6" s="120"/>
+      <c r="H6" s="120"/>
+      <c r="I6" s="120"/>
+      <c r="J6" s="120"/>
+      <c r="K6" s="120"/>
+      <c r="L6" s="120"/>
+      <c r="M6" s="120"/>
+      <c r="N6" s="120"/>
+      <c r="O6" s="120"/>
+      <c r="P6" s="120"/>
+      <c r="Q6" s="120"/>
+      <c r="R6" s="120"/>
+      <c r="S6" s="120"/>
+      <c r="T6" s="120"/>
+      <c r="U6" s="120"/>
+      <c r="V6" s="121"/>
+    </row>
+    <row r="7" spans="2:22">
+      <c r="B7" s="114"/>
+      <c r="C7" s="119"/>
+      <c r="D7" s="120"/>
+      <c r="E7" s="120"/>
+      <c r="F7" s="120"/>
+      <c r="G7" s="120"/>
+      <c r="H7" s="120"/>
+      <c r="I7" s="120"/>
+      <c r="J7" s="120"/>
+      <c r="K7" s="120"/>
+      <c r="L7" s="120"/>
+      <c r="M7" s="120"/>
+      <c r="N7" s="120"/>
+      <c r="O7" s="120"/>
+      <c r="P7" s="120"/>
+      <c r="Q7" s="120"/>
+      <c r="R7" s="120"/>
+      <c r="S7" s="120"/>
+      <c r="T7" s="120"/>
+      <c r="U7" s="120"/>
+      <c r="V7" s="121"/>
+    </row>
+    <row r="8" spans="2:22">
+      <c r="B8" s="114"/>
+      <c r="C8" s="119"/>
+      <c r="D8" s="120"/>
+      <c r="E8" s="120"/>
+      <c r="F8" s="120"/>
+      <c r="G8" s="120"/>
+      <c r="H8" s="120"/>
+      <c r="I8" s="120"/>
+      <c r="J8" s="120"/>
+      <c r="K8" s="120"/>
+      <c r="L8" s="120"/>
+      <c r="M8" s="120"/>
+      <c r="N8" s="120"/>
+      <c r="O8" s="120"/>
+      <c r="P8" s="120"/>
+      <c r="Q8" s="120"/>
+      <c r="R8" s="120"/>
+      <c r="S8" s="120"/>
+      <c r="T8" s="120"/>
+      <c r="U8" s="120"/>
+      <c r="V8" s="121"/>
+    </row>
+    <row r="9" spans="2:22">
+      <c r="B9" s="114"/>
+      <c r="C9" s="119"/>
+      <c r="D9" s="120"/>
+      <c r="E9" s="120"/>
+      <c r="F9" s="120"/>
+      <c r="G9" s="120"/>
+      <c r="H9" s="120"/>
+      <c r="I9" s="120"/>
+      <c r="J9" s="120"/>
+      <c r="K9" s="120"/>
+      <c r="L9" s="120"/>
+      <c r="M9" s="120"/>
+      <c r="N9" s="120"/>
+      <c r="O9" s="120"/>
+      <c r="P9" s="120"/>
+      <c r="Q9" s="120"/>
+      <c r="R9" s="120"/>
+      <c r="S9" s="120"/>
+      <c r="T9" s="120"/>
+      <c r="U9" s="120"/>
+      <c r="V9" s="121"/>
+    </row>
+    <row r="10" spans="2:22">
+      <c r="B10" s="114"/>
+      <c r="C10" s="119"/>
+      <c r="D10" s="120"/>
+      <c r="E10" s="120"/>
+      <c r="F10" s="120"/>
+      <c r="G10" s="120"/>
+      <c r="H10" s="120"/>
+      <c r="I10" s="120"/>
+      <c r="J10" s="120"/>
+      <c r="K10" s="120"/>
+      <c r="L10" s="120"/>
+      <c r="M10" s="120"/>
+      <c r="N10" s="120"/>
+      <c r="O10" s="120"/>
+      <c r="P10" s="120"/>
+      <c r="Q10" s="120"/>
+      <c r="R10" s="120"/>
+      <c r="S10" s="120"/>
+      <c r="T10" s="120"/>
+      <c r="U10" s="120"/>
+      <c r="V10" s="121"/>
+    </row>
+    <row r="11" spans="2:22">
+      <c r="B11" s="114"/>
+      <c r="C11" s="119"/>
+      <c r="D11" s="120"/>
+      <c r="E11" s="120"/>
+      <c r="F11" s="120"/>
+      <c r="G11" s="120"/>
+      <c r="H11" s="120"/>
+      <c r="I11" s="120"/>
+      <c r="J11" s="120"/>
+      <c r="K11" s="120"/>
+      <c r="L11" s="120"/>
+      <c r="M11" s="120"/>
+      <c r="N11" s="120"/>
+      <c r="O11" s="120"/>
+      <c r="P11" s="120"/>
+      <c r="Q11" s="120"/>
+      <c r="R11" s="120"/>
+      <c r="S11" s="120"/>
+      <c r="T11" s="120"/>
+      <c r="U11" s="120"/>
+      <c r="V11" s="121"/>
+    </row>
+    <row r="12" spans="2:22">
+      <c r="B12" s="114"/>
+      <c r="C12" s="119"/>
+      <c r="D12" s="120"/>
+      <c r="E12" s="120"/>
+      <c r="F12" s="120"/>
+      <c r="G12" s="120"/>
+      <c r="H12" s="120"/>
+      <c r="I12" s="120"/>
+      <c r="J12" s="120"/>
+      <c r="K12" s="120"/>
+      <c r="L12" s="120"/>
+      <c r="M12" s="120"/>
+      <c r="N12" s="120"/>
+      <c r="O12" s="120"/>
+      <c r="P12" s="120"/>
+      <c r="Q12" s="120"/>
+      <c r="R12" s="120"/>
+      <c r="S12" s="120"/>
+      <c r="T12" s="120"/>
+      <c r="U12" s="120"/>
+      <c r="V12" s="121"/>
+    </row>
+    <row r="13" spans="2:22" ht="14.25" thickBot="1">
+      <c r="B13" s="115"/>
+      <c r="C13" s="122"/>
+      <c r="D13" s="123"/>
+      <c r="E13" s="123"/>
+      <c r="F13" s="123"/>
+      <c r="G13" s="123"/>
+      <c r="H13" s="123"/>
+      <c r="I13" s="123"/>
+      <c r="J13" s="123"/>
+      <c r="K13" s="123"/>
+      <c r="L13" s="123"/>
+      <c r="M13" s="123"/>
+      <c r="N13" s="123"/>
+      <c r="O13" s="123"/>
+      <c r="P13" s="123"/>
+      <c r="Q13" s="123"/>
+      <c r="R13" s="123"/>
+      <c r="S13" s="123"/>
+      <c r="T13" s="123"/>
+      <c r="U13" s="123"/>
+      <c r="V13" s="124"/>
+    </row>
+    <row r="14" spans="2:22">
+      <c r="B14" s="113" t="s">
+        <v>154</v>
+      </c>
+      <c r="C14" s="125" t="s">
+        <v>151</v>
+      </c>
+      <c r="D14" s="126"/>
+      <c r="E14" s="126"/>
+      <c r="F14" s="126"/>
+      <c r="G14" s="126"/>
+      <c r="H14" s="126"/>
+      <c r="I14" s="126"/>
+      <c r="J14" s="126"/>
+      <c r="K14" s="126"/>
+      <c r="L14" s="126"/>
+      <c r="M14" s="126"/>
+      <c r="N14" s="126"/>
+      <c r="O14" s="126"/>
+      <c r="P14" s="126"/>
+      <c r="Q14" s="126"/>
+      <c r="R14" s="126"/>
+      <c r="S14" s="126"/>
+      <c r="T14" s="126"/>
+      <c r="U14" s="126"/>
+      <c r="V14" s="127"/>
+    </row>
+    <row r="15" spans="2:22">
+      <c r="B15" s="114"/>
+      <c r="C15" s="119"/>
+      <c r="D15" s="120"/>
+      <c r="E15" s="120"/>
+      <c r="F15" s="120"/>
+      <c r="G15" s="120"/>
+      <c r="H15" s="120"/>
+      <c r="I15" s="120"/>
+      <c r="J15" s="120"/>
+      <c r="K15" s="120"/>
+      <c r="L15" s="120"/>
+      <c r="M15" s="120"/>
+      <c r="N15" s="120"/>
+      <c r="O15" s="120"/>
+      <c r="P15" s="120"/>
+      <c r="Q15" s="120"/>
+      <c r="R15" s="120"/>
+      <c r="S15" s="120"/>
+      <c r="T15" s="120"/>
+      <c r="U15" s="120"/>
+      <c r="V15" s="121"/>
+    </row>
+    <row r="16" spans="2:22">
+      <c r="B16" s="114"/>
+      <c r="C16" s="119"/>
+      <c r="D16" s="120"/>
+      <c r="E16" s="120"/>
+      <c r="F16" s="120"/>
+      <c r="G16" s="120"/>
+      <c r="H16" s="120"/>
+      <c r="I16" s="120"/>
+      <c r="J16" s="120"/>
+      <c r="K16" s="120"/>
+      <c r="L16" s="120"/>
+      <c r="M16" s="120"/>
+      <c r="N16" s="120"/>
+      <c r="O16" s="120"/>
+      <c r="P16" s="120"/>
+      <c r="Q16" s="120"/>
+      <c r="R16" s="120"/>
+      <c r="S16" s="120"/>
+      <c r="T16" s="120"/>
+      <c r="U16" s="120"/>
+      <c r="V16" s="121"/>
+    </row>
+    <row r="17" spans="2:22">
+      <c r="B17" s="114"/>
+      <c r="C17" s="119"/>
+      <c r="D17" s="120"/>
+      <c r="E17" s="120"/>
+      <c r="F17" s="120"/>
+      <c r="G17" s="120"/>
+      <c r="H17" s="120"/>
+      <c r="I17" s="120"/>
+      <c r="J17" s="120"/>
+      <c r="K17" s="120"/>
+      <c r="L17" s="120"/>
+      <c r="M17" s="120"/>
+      <c r="N17" s="120"/>
+      <c r="O17" s="120"/>
+      <c r="P17" s="120"/>
+      <c r="Q17" s="120"/>
+      <c r="R17" s="120"/>
+      <c r="S17" s="120"/>
+      <c r="T17" s="120"/>
+      <c r="U17" s="120"/>
+      <c r="V17" s="121"/>
+    </row>
+    <row r="18" spans="2:22">
+      <c r="B18" s="114"/>
+      <c r="C18" s="119"/>
+      <c r="D18" s="120"/>
+      <c r="E18" s="120"/>
+      <c r="F18" s="120"/>
+      <c r="G18" s="120"/>
+      <c r="H18" s="120"/>
+      <c r="I18" s="120"/>
+      <c r="J18" s="120"/>
+      <c r="K18" s="120"/>
+      <c r="L18" s="120"/>
+      <c r="M18" s="120"/>
+      <c r="N18" s="120"/>
+      <c r="O18" s="120"/>
+      <c r="P18" s="120"/>
+      <c r="Q18" s="120"/>
+      <c r="R18" s="120"/>
+      <c r="S18" s="120"/>
+      <c r="T18" s="120"/>
+      <c r="U18" s="120"/>
+      <c r="V18" s="121"/>
+    </row>
+    <row r="19" spans="2:22">
+      <c r="B19" s="114"/>
+      <c r="C19" s="119"/>
+      <c r="D19" s="120"/>
+      <c r="E19" s="120"/>
+      <c r="F19" s="120"/>
+      <c r="G19" s="120"/>
+      <c r="H19" s="120"/>
+      <c r="I19" s="120"/>
+      <c r="J19" s="120"/>
+      <c r="K19" s="120"/>
+      <c r="L19" s="120"/>
+      <c r="M19" s="120"/>
+      <c r="N19" s="120"/>
+      <c r="O19" s="120"/>
+      <c r="P19" s="120"/>
+      <c r="Q19" s="120"/>
+      <c r="R19" s="120"/>
+      <c r="S19" s="120"/>
+      <c r="T19" s="120"/>
+      <c r="U19" s="120"/>
+      <c r="V19" s="121"/>
+    </row>
+    <row r="20" spans="2:22">
+      <c r="B20" s="114"/>
+      <c r="C20" s="119"/>
+      <c r="D20" s="120"/>
+      <c r="E20" s="120"/>
+      <c r="F20" s="120"/>
+      <c r="G20" s="120"/>
+      <c r="H20" s="120"/>
+      <c r="I20" s="120"/>
+      <c r="J20" s="120"/>
+      <c r="K20" s="120"/>
+      <c r="L20" s="120"/>
+      <c r="M20" s="120"/>
+      <c r="N20" s="120"/>
+      <c r="O20" s="120"/>
+      <c r="P20" s="120"/>
+      <c r="Q20" s="120"/>
+      <c r="R20" s="120"/>
+      <c r="S20" s="120"/>
+      <c r="T20" s="120"/>
+      <c r="U20" s="120"/>
+      <c r="V20" s="121"/>
+    </row>
+    <row r="21" spans="2:22">
+      <c r="B21" s="114"/>
+      <c r="C21" s="119"/>
+      <c r="D21" s="120"/>
+      <c r="E21" s="120"/>
+      <c r="F21" s="120"/>
+      <c r="G21" s="120"/>
+      <c r="H21" s="120"/>
+      <c r="I21" s="120"/>
+      <c r="J21" s="120"/>
+      <c r="K21" s="120"/>
+      <c r="L21" s="120"/>
+      <c r="M21" s="120"/>
+      <c r="N21" s="120"/>
+      <c r="O21" s="120"/>
+      <c r="P21" s="120"/>
+      <c r="Q21" s="120"/>
+      <c r="R21" s="120"/>
+      <c r="S21" s="120"/>
+      <c r="T21" s="120"/>
+      <c r="U21" s="120"/>
+      <c r="V21" s="121"/>
+    </row>
+    <row r="22" spans="2:22">
+      <c r="B22" s="114"/>
+      <c r="C22" s="119"/>
+      <c r="D22" s="120"/>
+      <c r="E22" s="120"/>
+      <c r="F22" s="120"/>
+      <c r="G22" s="120"/>
+      <c r="H22" s="120"/>
+      <c r="I22" s="120"/>
+      <c r="J22" s="120"/>
+      <c r="K22" s="120"/>
+      <c r="L22" s="120"/>
+      <c r="M22" s="120"/>
+      <c r="N22" s="120"/>
+      <c r="O22" s="120"/>
+      <c r="P22" s="120"/>
+      <c r="Q22" s="120"/>
+      <c r="R22" s="120"/>
+      <c r="S22" s="120"/>
+      <c r="T22" s="120"/>
+      <c r="U22" s="120"/>
+      <c r="V22" s="121"/>
+    </row>
+    <row r="23" spans="2:22">
+      <c r="B23" s="114"/>
+      <c r="C23" s="119"/>
+      <c r="D23" s="120"/>
+      <c r="E23" s="120"/>
+      <c r="F23" s="120"/>
+      <c r="G23" s="120"/>
+      <c r="H23" s="120"/>
+      <c r="I23" s="120"/>
+      <c r="J23" s="120"/>
+      <c r="K23" s="120"/>
+      <c r="L23" s="120"/>
+      <c r="M23" s="120"/>
+      <c r="N23" s="120"/>
+      <c r="O23" s="120"/>
+      <c r="P23" s="120"/>
+      <c r="Q23" s="120"/>
+      <c r="R23" s="120"/>
+      <c r="S23" s="120"/>
+      <c r="T23" s="120"/>
+      <c r="U23" s="120"/>
+      <c r="V23" s="121"/>
+    </row>
+    <row r="24" spans="2:22">
+      <c r="B24" s="114"/>
+      <c r="C24" s="119"/>
+      <c r="D24" s="120"/>
+      <c r="E24" s="120"/>
+      <c r="F24" s="120"/>
+      <c r="G24" s="120"/>
+      <c r="H24" s="120"/>
+      <c r="I24" s="120"/>
+      <c r="J24" s="120"/>
+      <c r="K24" s="120"/>
+      <c r="L24" s="120"/>
+      <c r="M24" s="120"/>
+      <c r="N24" s="120"/>
+      <c r="O24" s="120"/>
+      <c r="P24" s="120"/>
+      <c r="Q24" s="120"/>
+      <c r="R24" s="120"/>
+      <c r="S24" s="120"/>
+      <c r="T24" s="120"/>
+      <c r="U24" s="120"/>
+      <c r="V24" s="121"/>
+    </row>
+    <row r="25" spans="2:22" ht="14.25" thickBot="1">
+      <c r="B25" s="114"/>
+      <c r="C25" s="128"/>
+      <c r="D25" s="129"/>
+      <c r="E25" s="129"/>
+      <c r="F25" s="129"/>
+      <c r="G25" s="129"/>
+      <c r="H25" s="129"/>
+      <c r="I25" s="129"/>
+      <c r="J25" s="129"/>
+      <c r="K25" s="129"/>
+      <c r="L25" s="129"/>
+      <c r="M25" s="129"/>
+      <c r="N25" s="129"/>
+      <c r="O25" s="129"/>
+      <c r="P25" s="129"/>
+      <c r="Q25" s="129"/>
+      <c r="R25" s="129"/>
+      <c r="S25" s="129"/>
+      <c r="T25" s="129"/>
+      <c r="U25" s="129"/>
+      <c r="V25" s="130"/>
+    </row>
+    <row r="26" spans="2:22">
+      <c r="B26" s="113" t="s">
+        <v>153</v>
+      </c>
+      <c r="C26" s="116" t="s">
+        <v>152</v>
+      </c>
+      <c r="D26" s="117"/>
+      <c r="E26" s="117"/>
+      <c r="F26" s="117"/>
+      <c r="G26" s="117"/>
+      <c r="H26" s="117"/>
+      <c r="I26" s="117"/>
+      <c r="J26" s="117"/>
+      <c r="K26" s="117"/>
+      <c r="L26" s="117"/>
+      <c r="M26" s="117"/>
+      <c r="N26" s="117"/>
+      <c r="O26" s="117"/>
+      <c r="P26" s="117"/>
+      <c r="Q26" s="117"/>
+      <c r="R26" s="117"/>
+      <c r="S26" s="117"/>
+      <c r="T26" s="117"/>
+      <c r="U26" s="117"/>
+      <c r="V26" s="118"/>
+    </row>
+    <row r="27" spans="2:22">
+      <c r="B27" s="114"/>
+      <c r="C27" s="119"/>
+      <c r="D27" s="120"/>
+      <c r="E27" s="120"/>
+      <c r="F27" s="120"/>
+      <c r="G27" s="120"/>
+      <c r="H27" s="120"/>
+      <c r="I27" s="120"/>
+      <c r="J27" s="120"/>
+      <c r="K27" s="120"/>
+      <c r="L27" s="120"/>
+      <c r="M27" s="120"/>
+      <c r="N27" s="120"/>
+      <c r="O27" s="120"/>
+      <c r="P27" s="120"/>
+      <c r="Q27" s="120"/>
+      <c r="R27" s="120"/>
+      <c r="S27" s="120"/>
+      <c r="T27" s="120"/>
+      <c r="U27" s="120"/>
+      <c r="V27" s="121"/>
+    </row>
+    <row r="28" spans="2:22">
+      <c r="B28" s="114"/>
+      <c r="C28" s="119"/>
+      <c r="D28" s="120"/>
+      <c r="E28" s="120"/>
+      <c r="F28" s="120"/>
+      <c r="G28" s="120"/>
+      <c r="H28" s="120"/>
+      <c r="I28" s="120"/>
+      <c r="J28" s="120"/>
+      <c r="K28" s="120"/>
+      <c r="L28" s="120"/>
+      <c r="M28" s="120"/>
+      <c r="N28" s="120"/>
+      <c r="O28" s="120"/>
+      <c r="P28" s="120"/>
+      <c r="Q28" s="120"/>
+      <c r="R28" s="120"/>
+      <c r="S28" s="120"/>
+      <c r="T28" s="120"/>
+      <c r="U28" s="120"/>
+      <c r="V28" s="121"/>
+    </row>
+    <row r="29" spans="2:22">
+      <c r="B29" s="114"/>
+      <c r="C29" s="119"/>
+      <c r="D29" s="120"/>
+      <c r="E29" s="120"/>
+      <c r="F29" s="120"/>
+      <c r="G29" s="120"/>
+      <c r="H29" s="120"/>
+      <c r="I29" s="120"/>
+      <c r="J29" s="120"/>
+      <c r="K29" s="120"/>
+      <c r="L29" s="120"/>
+      <c r="M29" s="120"/>
+      <c r="N29" s="120"/>
+      <c r="O29" s="120"/>
+      <c r="P29" s="120"/>
+      <c r="Q29" s="120"/>
+      <c r="R29" s="120"/>
+      <c r="S29" s="120"/>
+      <c r="T29" s="120"/>
+      <c r="U29" s="120"/>
+      <c r="V29" s="121"/>
+    </row>
+    <row r="30" spans="2:22">
+      <c r="B30" s="114"/>
+      <c r="C30" s="119"/>
+      <c r="D30" s="120"/>
+      <c r="E30" s="120"/>
+      <c r="F30" s="120"/>
+      <c r="G30" s="120"/>
+      <c r="H30" s="120"/>
+      <c r="I30" s="120"/>
+      <c r="J30" s="120"/>
+      <c r="K30" s="120"/>
+      <c r="L30" s="120"/>
+      <c r="M30" s="120"/>
+      <c r="N30" s="120"/>
+      <c r="O30" s="120"/>
+      <c r="P30" s="120"/>
+      <c r="Q30" s="120"/>
+      <c r="R30" s="120"/>
+      <c r="S30" s="120"/>
+      <c r="T30" s="120"/>
+      <c r="U30" s="120"/>
+      <c r="V30" s="121"/>
+    </row>
+    <row r="31" spans="2:22">
+      <c r="B31" s="114"/>
+      <c r="C31" s="119"/>
+      <c r="D31" s="120"/>
+      <c r="E31" s="120"/>
+      <c r="F31" s="120"/>
+      <c r="G31" s="120"/>
+      <c r="H31" s="120"/>
+      <c r="I31" s="120"/>
+      <c r="J31" s="120"/>
+      <c r="K31" s="120"/>
+      <c r="L31" s="120"/>
+      <c r="M31" s="120"/>
+      <c r="N31" s="120"/>
+      <c r="O31" s="120"/>
+      <c r="P31" s="120"/>
+      <c r="Q31" s="120"/>
+      <c r="R31" s="120"/>
+      <c r="S31" s="120"/>
+      <c r="T31" s="120"/>
+      <c r="U31" s="120"/>
+      <c r="V31" s="121"/>
+    </row>
+    <row r="32" spans="2:22">
+      <c r="B32" s="114"/>
+      <c r="C32" s="119"/>
+      <c r="D32" s="120"/>
+      <c r="E32" s="120"/>
+      <c r="F32" s="120"/>
+      <c r="G32" s="120"/>
+      <c r="H32" s="120"/>
+      <c r="I32" s="120"/>
+      <c r="J32" s="120"/>
+      <c r="K32" s="120"/>
+      <c r="L32" s="120"/>
+      <c r="M32" s="120"/>
+      <c r="N32" s="120"/>
+      <c r="O32" s="120"/>
+      <c r="P32" s="120"/>
+      <c r="Q32" s="120"/>
+      <c r="R32" s="120"/>
+      <c r="S32" s="120"/>
+      <c r="T32" s="120"/>
+      <c r="U32" s="120"/>
+      <c r="V32" s="121"/>
+    </row>
+    <row r="33" spans="2:22">
+      <c r="B33" s="114"/>
+      <c r="C33" s="119"/>
+      <c r="D33" s="120"/>
+      <c r="E33" s="120"/>
+      <c r="F33" s="120"/>
+      <c r="G33" s="120"/>
+      <c r="H33" s="120"/>
+      <c r="I33" s="120"/>
+      <c r="J33" s="120"/>
+      <c r="K33" s="120"/>
+      <c r="L33" s="120"/>
+      <c r="M33" s="120"/>
+      <c r="N33" s="120"/>
+      <c r="O33" s="120"/>
+      <c r="P33" s="120"/>
+      <c r="Q33" s="120"/>
+      <c r="R33" s="120"/>
+      <c r="S33" s="120"/>
+      <c r="T33" s="120"/>
+      <c r="U33" s="120"/>
+      <c r="V33" s="121"/>
+    </row>
+    <row r="34" spans="2:22" ht="14.25" thickBot="1">
+      <c r="B34" s="115"/>
+      <c r="C34" s="128"/>
+      <c r="D34" s="129"/>
+      <c r="E34" s="129"/>
+      <c r="F34" s="129"/>
+      <c r="G34" s="129"/>
+      <c r="H34" s="129"/>
+      <c r="I34" s="129"/>
+      <c r="J34" s="129"/>
+      <c r="K34" s="129"/>
+      <c r="L34" s="129"/>
+      <c r="M34" s="129"/>
+      <c r="N34" s="129"/>
+      <c r="O34" s="129"/>
+      <c r="P34" s="129"/>
+      <c r="Q34" s="129"/>
+      <c r="R34" s="129"/>
+      <c r="S34" s="129"/>
+      <c r="T34" s="129"/>
+      <c r="U34" s="129"/>
+      <c r="V34" s="130"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="H2:N2"/>
+    <mergeCell ref="B4:B13"/>
+    <mergeCell ref="C4:V13"/>
+    <mergeCell ref="B14:B25"/>
+    <mergeCell ref="C14:V25"/>
+    <mergeCell ref="B26:B34"/>
+    <mergeCell ref="C26:V34"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>